<commit_message>
fixed issue with translational sector config
</commit_message>
<xml_diff>
--- a/Data/Pputida_phenotypes/pputida_phenotypes.xlsx
+++ b/Data/Pputida_phenotypes/pputida_phenotypes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="257" uniqueCount="125">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="122">
   <si>
     <t xml:space="preserve">exchanges</t>
   </si>
@@ -119,6 +119,9 @@
     <t xml:space="preserve">Fluxomics datasets in mmol/g_cdw/h</t>
   </si>
   <si>
+    <t xml:space="preserve">Fructose fluxomics data is possibly mixotrophic growth, could not find exclusion from paper</t>
+  </si>
+  <si>
     <t xml:space="preserve">EX_glcn_e</t>
   </si>
   <si>
@@ -131,7 +134,7 @@
     <t xml:space="preserve">Info</t>
   </si>
   <si>
-    <t xml:space="preserve">P. putida KT2440</t>
+    <t xml:space="preserve">KT2440</t>
   </si>
   <si>
     <t xml:space="preserve">10.1128/AEM.05588-11</t>
@@ -140,19 +143,16 @@
     <t xml:space="preserve">Empty pCOM10 expressed</t>
   </si>
   <si>
-    <t xml:space="preserve">P. putida Gpo12</t>
+    <t xml:space="preserve">Gpo12</t>
   </si>
   <si>
     <t xml:space="preserve">10.1111/j.1742-4658.2008.06648.x</t>
   </si>
   <si>
-    <t xml:space="preserve">P. putida S12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P. putida DOT-T1E</t>
-  </si>
-  <si>
-    <t xml:space="preserve">KT2440</t>
+    <t xml:space="preserve">S12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DOT-T1E</t>
   </si>
   <si>
     <t xml:space="preserve">10.1128/JB.00203-07</t>
@@ -170,12 +170,6 @@
     <t xml:space="preserve">pWW0 plasmid for toluene degradation. the gluconate and ketogluconate is not specify so the net carbon uptake might differ</t>
   </si>
   <si>
-    <t xml:space="preserve">Gpo12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S12</t>
-  </si>
-  <si>
     <t xml:space="preserve">10.1002/elsc.201600072</t>
   </si>
   <si>
@@ -378,9 +372,6 @@
   </si>
   <si>
     <t xml:space="preserve">10.1111/j.1742-4658.2008.06648.x (S12)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">AEM.01643-14 (glucose)</t>
   </si>
   <si>
     <t xml:space="preserve">10.1002/elsc.201600072 (batch)</t>
@@ -668,8 +659,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:M10"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:M11"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -803,6 +794,11 @@
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="8" t="s">
         <v>30</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -822,7 +818,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AMJ36"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
@@ -832,7 +828,7 @@
         <v>5</v>
       </c>
       <c r="C1" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D1" s="9" t="s">
         <v>7</v>
@@ -856,13 +852,13 @@
         <v>14</v>
       </c>
       <c r="K1" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="L1" s="8" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="M1" s="8" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="AMJ1" s="0"/>
     </row>
@@ -882,10 +878,10 @@
       <c r="I2" s="10"/>
       <c r="J2" s="10"/>
       <c r="K2" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L2" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -904,13 +900,13 @@
       <c r="I3" s="10"/>
       <c r="J3" s="10"/>
       <c r="K3" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L3" s="11" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -933,10 +929,10 @@
       <c r="I4" s="10"/>
       <c r="J4" s="10"/>
       <c r="K4" s="10" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -959,10 +955,10 @@
       <c r="I5" s="10"/>
       <c r="J5" s="10"/>
       <c r="K5" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -985,10 +981,10 @@
       <c r="I6" s="10"/>
       <c r="J6" s="10"/>
       <c r="K6" s="10" t="s">
+        <v>41</v>
+      </c>
+      <c r="L6" s="2" t="s">
         <v>40</v>
-      </c>
-      <c r="L6" s="2" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1011,10 +1007,10 @@
       <c r="I7" s="10"/>
       <c r="J7" s="10"/>
       <c r="K7" s="10" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1037,7 +1033,7 @@
       <c r="I8" s="10"/>
       <c r="J8" s="10"/>
       <c r="K8" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>43</v>
@@ -1063,7 +1059,7 @@
       <c r="I9" s="10"/>
       <c r="J9" s="10"/>
       <c r="K9" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>44</v>
@@ -1085,7 +1081,7 @@
       <c r="I10" s="10"/>
       <c r="J10" s="10"/>
       <c r="K10" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>44</v>
@@ -1163,10 +1159,10 @@
       <c r="I13" s="10"/>
       <c r="J13" s="10"/>
       <c r="K13" s="12" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1189,10 +1185,10 @@
       <c r="I14" s="10"/>
       <c r="J14" s="10"/>
       <c r="K14" s="12" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1215,10 +1211,10 @@
       <c r="I15" s="10"/>
       <c r="J15" s="10"/>
       <c r="K15" s="12" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1237,13 +1233,13 @@
       <c r="I16" s="10"/>
       <c r="J16" s="10"/>
       <c r="K16" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1262,13 +1258,13 @@
       <c r="I17" s="10"/>
       <c r="J17" s="10"/>
       <c r="K17" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L17" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="M17" s="2" t="s">
         <v>50</v>
-      </c>
-      <c r="M17" s="2" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1287,10 +1283,10 @@
       <c r="I18" s="10"/>
       <c r="J18" s="10"/>
       <c r="K18" s="10" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="L18" s="2" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1310,13 +1306,13 @@
       <c r="I19" s="10"/>
       <c r="J19" s="10"/>
       <c r="K19" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L19" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M19" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1336,13 +1332,13 @@
       <c r="I20" s="10"/>
       <c r="J20" s="10"/>
       <c r="K20" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L20" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M20" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1362,13 +1358,13 @@
       <c r="I21" s="10"/>
       <c r="J21" s="10"/>
       <c r="K21" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L21" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M21" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1388,13 +1384,13 @@
       <c r="I22" s="10"/>
       <c r="J22" s="10"/>
       <c r="K22" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L22" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M22" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1414,13 +1410,13 @@
       <c r="I23" s="10"/>
       <c r="J23" s="10"/>
       <c r="K23" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L23" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M23" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1440,13 +1436,13 @@
       <c r="I24" s="10"/>
       <c r="J24" s="10"/>
       <c r="K24" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L24" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M24" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1466,13 +1462,13 @@
       <c r="I25" s="10"/>
       <c r="J25" s="10"/>
       <c r="K25" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L25" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M25" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1492,13 +1488,13 @@
       <c r="I26" s="10"/>
       <c r="J26" s="10"/>
       <c r="K26" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L26" s="2" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="M26" s="2" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1520,7 +1516,7 @@
         <v>45</v>
       </c>
       <c r="L27" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1542,7 +1538,7 @@
         <v>45</v>
       </c>
       <c r="L28" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1564,7 +1560,7 @@
         <v>45</v>
       </c>
       <c r="L29" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1586,7 +1582,7 @@
         <v>45</v>
       </c>
       <c r="L30" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1608,7 +1604,7 @@
         <v>45</v>
       </c>
       <c r="L31" s="11" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1627,13 +1623,13 @@
       <c r="I32" s="10"/>
       <c r="J32" s="10"/>
       <c r="K32" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L32" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="M32" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="L32" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="M32" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1652,13 +1648,13 @@
       </c>
       <c r="J33" s="10"/>
       <c r="K33" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="L33" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="M33" s="2" t="s">
         <v>58</v>
-      </c>
-      <c r="L33" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="M33" s="2" t="s">
-        <v>60</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1677,10 +1673,10 @@
       <c r="I34" s="10"/>
       <c r="J34" s="10"/>
       <c r="K34" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L34" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1699,10 +1695,10 @@
       <c r="I35" s="10"/>
       <c r="J35" s="10"/>
       <c r="K35" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L35" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1721,10 +1717,10 @@
       <c r="I36" s="10"/>
       <c r="J36" s="10"/>
       <c r="K36" s="10" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="L36" s="2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
     </row>
   </sheetData>
@@ -1743,116 +1739,119 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AJ3"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AK3"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B1" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="C1" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="D1" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="E1" s="8" t="s">
         <v>64</v>
       </c>
-      <c r="D1" s="8" t="s">
+      <c r="F1" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="E1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>66</v>
       </c>
-      <c r="F1" s="8" t="s">
+      <c r="H1" s="8" t="s">
         <v>67</v>
       </c>
-      <c r="G1" s="8" t="s">
+      <c r="I1" s="8" t="s">
         <v>68</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="J1" s="8" t="s">
         <v>69</v>
       </c>
-      <c r="I1" s="8" t="s">
+      <c r="K1" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>71</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="L1" s="8" t="s">
+      <c r="N1" s="8" t="s">
         <v>73</v>
       </c>
-      <c r="M1" s="8" t="s">
+      <c r="O1" s="8" t="s">
         <v>74</v>
       </c>
-      <c r="N1" s="8" t="s">
+      <c r="P1" s="8" t="s">
         <v>75</v>
       </c>
-      <c r="O1" s="8" t="s">
+      <c r="Q1" s="8" t="s">
         <v>76</v>
       </c>
-      <c r="P1" s="8" t="s">
+      <c r="R1" s="8" t="s">
         <v>77</v>
       </c>
-      <c r="Q1" s="8" t="s">
+      <c r="S1" s="8" t="s">
         <v>78</v>
       </c>
-      <c r="R1" s="8" t="s">
+      <c r="T1" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="S1" s="8" t="s">
+      <c r="U1" s="8" t="s">
         <v>80</v>
       </c>
-      <c r="T1" s="8" t="s">
+      <c r="V1" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="U1" s="8" t="s">
+      <c r="W1" s="8" t="s">
         <v>82</v>
       </c>
-      <c r="V1" s="8" t="s">
+      <c r="X1" s="8" t="s">
         <v>83</v>
       </c>
-      <c r="W1" s="8" t="s">
+      <c r="Y1" s="8" t="s">
         <v>84</v>
       </c>
-      <c r="X1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="Y1" s="8" t="s">
+      <c r="AA1" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="Z1" s="8" t="s">
+      <c r="AB1" s="8" t="s">
         <v>87</v>
       </c>
-      <c r="AA1" s="8" t="s">
+      <c r="AC1" s="8" t="s">
         <v>88</v>
       </c>
-      <c r="AB1" s="8" t="s">
+      <c r="AD1" s="8" t="s">
         <v>89</v>
       </c>
-      <c r="AC1" s="8" t="s">
+      <c r="AE1" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="AD1" s="8" t="s">
+      <c r="AF1" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="AE1" s="8" t="s">
+      <c r="AG1" s="8" t="s">
         <v>92</v>
       </c>
-      <c r="AF1" s="8" t="s">
+      <c r="AH1" s="8" t="s">
         <v>93</v>
-      </c>
-      <c r="AG1" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="AH1" s="8" t="s">
-        <v>95</v>
       </c>
       <c r="AI1" s="8" t="s">
         <v>4</v>
       </c>
       <c r="AJ1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AK1" s="8" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1963,7 +1962,10 @@
         <v>0.2</v>
       </c>
       <c r="AJ2" s="11" t="s">
-        <v>96</v>
+        <v>94</v>
+      </c>
+      <c r="AK2" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2060,8 +2062,14 @@
       <c r="AG3" s="2" t="n">
         <v>0.05</v>
       </c>
+      <c r="AI3" s="0" t="n">
+        <v>0.1</v>
+      </c>
       <c r="AJ3" s="2" t="s">
-        <v>97</v>
+        <v>95</v>
+      </c>
+      <c r="AK3" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2080,131 +2088,137 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AO8"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AQ7"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
         <v>5</v>
       </c>
       <c r="B1" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>97</v>
+      </c>
+      <c r="D1" s="16" t="s">
         <v>98</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="E1" s="17" t="s">
         <v>99</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="F1" s="17" t="s">
         <v>100</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="G1" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="H1" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="I1" s="16" t="s">
+        <v>88</v>
+      </c>
+      <c r="J1" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="K1" s="18" t="s">
+        <v>90</v>
+      </c>
+      <c r="L1" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="M1" s="17" t="s">
         <v>104</v>
       </c>
-      <c r="I1" s="16" t="s">
-        <v>90</v>
-      </c>
-      <c r="J1" s="17" t="s">
+      <c r="N1" s="17" t="s">
+        <v>105</v>
+      </c>
+      <c r="O1" s="17" t="s">
+        <v>106</v>
+      </c>
+      <c r="P1" s="17" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q1" s="17" t="s">
+        <v>108</v>
+      </c>
+      <c r="R1" s="17" t="s">
+        <v>93</v>
+      </c>
+      <c r="S1" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="T1" s="18" t="s">
         <v>92</v>
       </c>
-      <c r="L1" s="16" t="s">
-        <v>105</v>
-      </c>
-      <c r="M1" s="17" t="s">
-        <v>106</v>
-      </c>
-      <c r="N1" s="17" t="s">
-        <v>107</v>
-      </c>
-      <c r="O1" s="17" t="s">
-        <v>108</v>
-      </c>
-      <c r="P1" s="17" t="s">
+      <c r="U1" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="V1" s="17" t="s">
+        <v>85</v>
+      </c>
+      <c r="W1" s="17" t="s">
+        <v>84</v>
+      </c>
+      <c r="X1" s="17" t="s">
+        <v>83</v>
+      </c>
+      <c r="Y1" s="18" t="s">
         <v>109</v>
       </c>
-      <c r="Q1" s="17" t="s">
+      <c r="Z1" s="16" t="s">
+        <v>77</v>
+      </c>
+      <c r="AA1" s="17" t="s">
+        <v>69</v>
+      </c>
+      <c r="AB1" s="17" t="s">
         <v>110</v>
       </c>
-      <c r="R1" s="17" t="s">
-        <v>95</v>
-      </c>
-      <c r="S1" s="18" t="s">
-        <v>93</v>
-      </c>
-      <c r="T1" s="18" t="s">
-        <v>94</v>
-      </c>
-      <c r="U1" s="16" t="s">
-        <v>88</v>
-      </c>
-      <c r="V1" s="17" t="s">
-        <v>87</v>
-      </c>
-      <c r="W1" s="17" t="s">
-        <v>86</v>
-      </c>
-      <c r="X1" s="17" t="s">
-        <v>85</v>
-      </c>
-      <c r="Y1" s="18" t="s">
+      <c r="AC1" s="17" t="s">
+        <v>76</v>
+      </c>
+      <c r="AD1" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="AE1" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="AF1" s="17" t="s">
+        <v>78</v>
+      </c>
+      <c r="AG1" s="17" t="s">
+        <v>79</v>
+      </c>
+      <c r="AH1" s="17" t="s">
+        <v>80</v>
+      </c>
+      <c r="AI1" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="AJ1" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="AK1" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="AL1" s="8" t="s">
         <v>111</v>
       </c>
-      <c r="Z1" s="16" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA1" s="17" t="s">
-        <v>71</v>
-      </c>
-      <c r="AB1" s="17" t="s">
+      <c r="AM1" s="8" t="s">
+        <v>81</v>
+      </c>
+      <c r="AN1" s="8" t="s">
         <v>112</v>
       </c>
-      <c r="AC1" s="17" t="s">
-        <v>78</v>
-      </c>
-      <c r="AD1" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="AE1" s="17" t="s">
-        <v>73</v>
-      </c>
-      <c r="AF1" s="17" t="s">
-        <v>80</v>
-      </c>
-      <c r="AG1" s="17" t="s">
-        <v>81</v>
-      </c>
-      <c r="AH1" s="17" t="s">
-        <v>82</v>
-      </c>
-      <c r="AI1" s="17" t="s">
-        <v>75</v>
-      </c>
-      <c r="AJ1" s="17" t="s">
-        <v>76</v>
-      </c>
-      <c r="AK1" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="AL1" s="8" t="s">
-        <v>113</v>
-      </c>
-      <c r="AM1" s="8" t="s">
-        <v>83</v>
-      </c>
-      <c r="AN1" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="AO1" s="8" t="s">
+      <c r="AO1" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="AP1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AQ1" s="8" t="s">
         <v>33</v>
       </c>
     </row>
@@ -2358,8 +2372,14 @@
         <f aca="false">44/100*6.14</f>
         <v>2.7016</v>
       </c>
-      <c r="AO2" s="11" t="s">
+      <c r="AO2" s="0" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="AP2" s="11" t="s">
         <v>44</v>
+      </c>
+      <c r="AQ2" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2455,8 +2475,14 @@
         <f aca="false">10/100*5.7</f>
         <v>0.57</v>
       </c>
-      <c r="AO3" s="11" t="s">
-        <v>115</v>
+      <c r="AO3" s="0" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AP3" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="AQ3" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2553,8 +2579,14 @@
         <f aca="false">18/100*5.2</f>
         <v>0.936</v>
       </c>
-      <c r="AO4" s="11" t="s">
-        <v>116</v>
+      <c r="AO4" s="0" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="AP4" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="AQ4" s="0" t="s">
+        <v>39</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2651,320 +2683,255 @@
         <f aca="false">16/100*6.5</f>
         <v>1.04</v>
       </c>
-      <c r="AO5" s="11" t="s">
-        <v>117</v>
+      <c r="AO5" s="0" t="n">
+        <v>0.52</v>
+      </c>
+      <c r="AP5" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="AQ5" s="0" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="n">
-        <v>-2.21</v>
-      </c>
-      <c r="D6" s="2" t="n">
-        <v>2.21</v>
+        <v>-6.01</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>2.2</v>
+        <f aca="false">99/100*6.01</f>
+        <v>5.9499</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>2.2</v>
+        <f aca="false">99/100*6.01</f>
+        <v>5.9499</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>2.14</v>
+        <f aca="false">94/100*6.01</f>
+        <v>5.6494</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>2.14</v>
+        <f aca="false">94/100*6.01</f>
+        <v>5.6494</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="O6" s="2" t="n">
-        <v>0.06</v>
+        <f aca="false">6/100*6.01</f>
+        <v>0.3606</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>0.01</v>
+        <v>0</v>
+      </c>
+      <c r="T6" s="2" t="n">
+        <f aca="false">-4/100*6.01</f>
+        <v>-0.2404</v>
       </c>
       <c r="U6" s="2" t="n">
-        <v>2.13</v>
+        <f aca="false">80/100*6.01</f>
+        <v>4.808</v>
       </c>
       <c r="V6" s="2" t="n">
-        <v>2.13</v>
+        <f aca="false">80/100*6.01</f>
+        <v>4.808</v>
       </c>
       <c r="W6" s="2" t="n">
-        <v>1.96</v>
+        <f aca="false">80/100*6.01</f>
+        <v>4.808</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>1.96</v>
+        <f aca="false">80/100*6.01</f>
+        <v>4.808</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>2.21</v>
+        <f aca="false">54/100*6.01</f>
+        <v>3.2454</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>3.23</v>
+        <f aca="false">87/100*6.01</f>
+        <v>5.2287</v>
+      </c>
+      <c r="AA6" s="2" t="n">
+        <f aca="false">63/100*6.01</f>
+        <v>3.7863</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>0.73</v>
+        <f aca="false">80/100*6.01</f>
+        <v>4.808</v>
       </c>
       <c r="AD6" s="2" t="n">
-        <v>2.98</v>
+        <f aca="false">63/100*6.01</f>
+        <v>3.7863</v>
       </c>
       <c r="AE6" s="2" t="n">
-        <v>2.98</v>
+        <f aca="false">63/100*6.01</f>
+        <v>3.7863</v>
       </c>
       <c r="AF6" s="2" t="n">
-        <v>2.98</v>
+        <f aca="false">63/100*6.01</f>
+        <v>3.7863</v>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>2.8</v>
+        <f aca="false">50/100*6.01</f>
+        <v>3.005</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>2.8</v>
+        <f aca="false">50/100*6.01</f>
+        <v>3.005</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>2.8</v>
+        <f aca="false">50/100*6.01</f>
+        <v>3.005</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>2.8</v>
+        <f aca="false">50/100*6.01</f>
+        <v>3.005</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="AM6" s="2" t="n">
-        <v>3.48</v>
-      </c>
-      <c r="AN6" s="2" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="AO6" s="11" t="s">
-        <v>118</v>
+        <v>0</v>
+      </c>
+      <c r="AL6" s="2" t="n">
+        <f aca="false">50/100*6.01</f>
+        <v>3.005</v>
+      </c>
+      <c r="AO6" s="0" t="n">
+        <v>0.61</v>
+      </c>
+      <c r="AP6" s="11" t="s">
+        <v>116</v>
+      </c>
+      <c r="AQ6" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="2" t="n">
-        <v>-6.01</v>
+        <v>-2.01</v>
       </c>
       <c r="E7" s="2" t="n">
-        <f aca="false">99/100*6.01</f>
-        <v>5.9499</v>
+        <f aca="false">98/100*2.01</f>
+        <v>1.9698</v>
       </c>
       <c r="F7" s="2" t="n">
-        <f aca="false">99/100*6.01</f>
-        <v>5.9499</v>
+        <f aca="false">98/100*2.01</f>
+        <v>1.9698</v>
       </c>
       <c r="G7" s="2" t="n">
-        <f aca="false">94/100*6.01</f>
-        <v>5.6494</v>
+        <f aca="false">98/100*2.01</f>
+        <v>1.9698</v>
       </c>
       <c r="H7" s="2" t="n">
-        <f aca="false">94/100*6.01</f>
-        <v>5.6494</v>
+        <f aca="false">98/100*2.01</f>
+        <v>1.9698</v>
       </c>
       <c r="I7" s="2" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="O7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K7" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="2" t="n">
-        <f aca="false">6/100*6.01</f>
-        <v>0.3606</v>
-      </c>
       <c r="R7" s="2" t="n">
-        <v>0</v>
+        <f aca="false">-2/100*2.01</f>
+        <v>-0.0402</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>0</v>
+        <f aca="false">-2/100*2.01</f>
+        <v>-0.0402</v>
       </c>
       <c r="T7" s="2" t="n">
-        <f aca="false">-4/100*6.01</f>
-        <v>-0.2404</v>
+        <f aca="false">-5/100*2.01</f>
+        <v>-0.1005</v>
       </c>
       <c r="U7" s="2" t="n">
-        <f aca="false">80/100*6.01</f>
-        <v>4.808</v>
+        <f aca="false">78/100*2.01</f>
+        <v>1.5678</v>
       </c>
       <c r="V7" s="2" t="n">
-        <f aca="false">80/100*6.01</f>
-        <v>4.808</v>
+        <f aca="false">78/100*2.01</f>
+        <v>1.5678</v>
       </c>
       <c r="W7" s="2" t="n">
-        <f aca="false">80/100*6.01</f>
-        <v>4.808</v>
+        <f aca="false">78/100*2.01</f>
+        <v>1.5678</v>
       </c>
       <c r="X7" s="2" t="n">
-        <f aca="false">80/100*6.01</f>
-        <v>4.808</v>
+        <f aca="false">78/100*2.01</f>
+        <v>1.5678</v>
       </c>
       <c r="Y7" s="2" t="n">
-        <f aca="false">54/100*6.01</f>
-        <v>3.2454</v>
+        <f aca="false">52/100*2.01</f>
+        <v>1.0452</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <f aca="false">87/100*6.01</f>
-        <v>5.2287</v>
+        <f aca="false">90/100*2.01</f>
+        <v>1.809</v>
       </c>
       <c r="AA7" s="2" t="n">
-        <f aca="false">63/100*6.01</f>
-        <v>3.7863</v>
+        <f aca="false">67/100*2.01</f>
+        <v>1.3467</v>
       </c>
       <c r="AB7" s="2" t="n">
-        <f aca="false">80/100*6.01</f>
-        <v>4.808</v>
+        <f aca="false">84/100*2.01</f>
+        <v>1.6884</v>
       </c>
       <c r="AD7" s="2" t="n">
-        <f aca="false">63/100*6.01</f>
-        <v>3.7863</v>
+        <f aca="false">67/100*2.01</f>
+        <v>1.3467</v>
       </c>
       <c r="AE7" s="2" t="n">
-        <f aca="false">63/100*6.01</f>
-        <v>3.7863</v>
+        <f aca="false">67/100*2.01</f>
+        <v>1.3467</v>
       </c>
       <c r="AF7" s="2" t="n">
-        <f aca="false">63/100*6.01</f>
-        <v>3.7863</v>
+        <f aca="false">67/100*2.01</f>
+        <v>1.3467</v>
       </c>
       <c r="AG7" s="2" t="n">
-        <f aca="false">50/100*6.01</f>
-        <v>3.005</v>
+        <f aca="false">54/100*2.01</f>
+        <v>1.0854</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <f aca="false">50/100*6.01</f>
-        <v>3.005</v>
+        <f aca="false">54/100*2.01</f>
+        <v>1.0854</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <f aca="false">50/100*6.01</f>
-        <v>3.005</v>
+        <f aca="false">54/100*2.01</f>
+        <v>1.0854</v>
       </c>
       <c r="AJ7" s="2" t="n">
-        <f aca="false">50/100*6.01</f>
-        <v>3.005</v>
+        <f aca="false">54/100*2.01</f>
+        <v>1.0854</v>
       </c>
       <c r="AK7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <f aca="false">50/100*6.01</f>
-        <v>3.005</v>
-      </c>
-      <c r="AO7" s="11" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="n">
-        <v>-2.01</v>
-      </c>
-      <c r="E8" s="2" t="n">
-        <f aca="false">98/100*2.01</f>
-        <v>1.9698</v>
-      </c>
-      <c r="F8" s="2" t="n">
-        <f aca="false">98/100*2.01</f>
-        <v>1.9698</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <f aca="false">98/100*2.01</f>
-        <v>1.9698</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <f aca="false">98/100*2.01</f>
-        <v>1.9698</v>
-      </c>
-      <c r="I8" s="2" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="K8" s="2" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="O8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R8" s="2" t="n">
-        <f aca="false">-2/100*2.01</f>
-        <v>-0.0402</v>
-      </c>
-      <c r="S8" s="2" t="n">
-        <f aca="false">-2/100*2.01</f>
-        <v>-0.0402</v>
-      </c>
-      <c r="T8" s="2" t="n">
-        <f aca="false">-5/100*2.01</f>
-        <v>-0.1005</v>
-      </c>
-      <c r="U8" s="2" t="n">
-        <f aca="false">78/100*2.01</f>
-        <v>1.5678</v>
-      </c>
-      <c r="V8" s="2" t="n">
-        <f aca="false">78/100*2.01</f>
-        <v>1.5678</v>
-      </c>
-      <c r="W8" s="2" t="n">
-        <f aca="false">78/100*2.01</f>
-        <v>1.5678</v>
-      </c>
-      <c r="X8" s="2" t="n">
-        <f aca="false">78/100*2.01</f>
-        <v>1.5678</v>
-      </c>
-      <c r="Y8" s="2" t="n">
-        <f aca="false">52/100*2.01</f>
-        <v>1.0452</v>
-      </c>
-      <c r="Z8" s="2" t="n">
-        <f aca="false">90/100*2.01</f>
-        <v>1.809</v>
-      </c>
-      <c r="AA8" s="2" t="n">
-        <f aca="false">67/100*2.01</f>
-        <v>1.3467</v>
-      </c>
-      <c r="AB8" s="2" t="n">
-        <f aca="false">84/100*2.01</f>
-        <v>1.6884</v>
-      </c>
-      <c r="AD8" s="2" t="n">
-        <f aca="false">67/100*2.01</f>
-        <v>1.3467</v>
-      </c>
-      <c r="AE8" s="2" t="n">
-        <f aca="false">67/100*2.01</f>
-        <v>1.3467</v>
-      </c>
-      <c r="AF8" s="2" t="n">
-        <f aca="false">67/100*2.01</f>
-        <v>1.3467</v>
-      </c>
-      <c r="AG8" s="2" t="n">
         <f aca="false">54/100*2.01</f>
         <v>1.0854</v>
       </c>
-      <c r="AH8" s="2" t="n">
-        <f aca="false">54/100*2.01</f>
-        <v>1.0854</v>
-      </c>
-      <c r="AI8" s="2" t="n">
-        <f aca="false">54/100*2.01</f>
-        <v>1.0854</v>
-      </c>
-      <c r="AJ8" s="2" t="n">
-        <f aca="false">54/100*2.01</f>
-        <v>1.0854</v>
-      </c>
-      <c r="AK8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL8" s="2" t="n">
-        <f aca="false">54/100*2.01</f>
-        <v>1.0854</v>
-      </c>
-      <c r="AO8" s="11" t="s">
-        <v>120</v>
+      <c r="AO7" s="0" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AP7" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="AQ7" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -2983,104 +2950,107 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AF2"/>
-  <sheetFormatPr defaultColWidth="11.5703125" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AG2"/>
+  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
         <v>13</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E1" s="8" t="s">
+        <v>89</v>
+      </c>
+      <c r="F1" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="G1" s="8" t="s">
+        <v>99</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>100</v>
+      </c>
+      <c r="I1" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>93</v>
+      </c>
+      <c r="K1" s="8" t="s">
         <v>91</v>
       </c>
-      <c r="F1" s="8" t="s">
-        <v>92</v>
-      </c>
-      <c r="G1" s="8" t="s">
+      <c r="L1" s="8" t="s">
         <v>101</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="M1" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="I1" s="8" t="s">
-        <v>108</v>
-      </c>
-      <c r="J1" s="8" t="s">
-        <v>95</v>
-      </c>
-      <c r="K1" s="8" t="s">
-        <v>93</v>
-      </c>
-      <c r="L1" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="M1" s="8" t="s">
-        <v>104</v>
-      </c>
       <c r="N1" s="8" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="O1" s="8" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="P1" s="8" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="R1" s="8" t="s">
+        <v>77</v>
+      </c>
+      <c r="S1" s="8" t="s">
+        <v>110</v>
+      </c>
+      <c r="T1" s="8" t="s">
+        <v>112</v>
+      </c>
+      <c r="U1" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="V1" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="W1" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="X1" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="Y1" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="S1" s="8" t="s">
-        <v>112</v>
-      </c>
-      <c r="T1" s="8" t="s">
-        <v>114</v>
-      </c>
-      <c r="U1" s="8" t="s">
-        <v>71</v>
-      </c>
-      <c r="V1" s="8" t="s">
+      <c r="Z1" s="8" t="s">
+        <v>80</v>
+      </c>
+      <c r="AA1" s="8" t="s">
+        <v>73</v>
+      </c>
+      <c r="AB1" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="AC1" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="AD1" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="W1" s="8" t="s">
-        <v>73</v>
-      </c>
-      <c r="X1" s="8" t="s">
-        <v>80</v>
-      </c>
-      <c r="Y1" s="8" t="s">
+      <c r="AE1" s="8" t="s">
         <v>81</v>
       </c>
-      <c r="Z1" s="8" t="s">
-        <v>82</v>
-      </c>
-      <c r="AA1" s="8" t="s">
-        <v>75</v>
-      </c>
-      <c r="AB1" s="8" t="s">
-        <v>76</v>
-      </c>
-      <c r="AC1" s="8" t="s">
-        <v>77</v>
-      </c>
-      <c r="AD1" s="8" t="s">
-        <v>74</v>
-      </c>
-      <c r="AE1" s="8" t="s">
-        <v>83</v>
-      </c>
       <c r="AF1" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="AG1" s="8" t="s">
         <v>33</v>
       </c>
     </row>
@@ -3179,7 +3149,10 @@
         <v>1.82</v>
       </c>
       <c r="AF2" s="2" t="s">
-        <v>124</v>
+        <v>121</v>
+      </c>
+      <c r="AG2" s="0" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
made sure unit tests pass. Improved robustness
</commit_message>
<xml_diff>
--- a/Data/Pputida_phenotypes/pputida_phenotypes.xlsx
+++ b/Data/Pputida_phenotypes/pputida_phenotypes.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId2"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="122">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="122">
   <si>
     <t xml:space="preserve">exchanges</t>
   </si>
@@ -125,6 +125,9 @@
     <t xml:space="preserve">EX_glcn_e</t>
   </si>
   <si>
+    <t xml:space="preserve">EX_bz_e</t>
+  </si>
+  <si>
     <t xml:space="preserve">Strain</t>
   </si>
   <si>
@@ -179,9 +182,6 @@
     <t xml:space="preserve">Chemostat experiment. Glucose uptake rate is the sum of glucose,gluconate, and 2-ketogluconate</t>
   </si>
   <si>
-    <t xml:space="preserve">KT2442</t>
-  </si>
-  <si>
     <t xml:space="preserve">10.1111/j.1462-2920.2011.02684.x</t>
   </si>
   <si>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">10.1111/1462-2920.12224</t>
   </si>
   <si>
-    <t xml:space="preserve">EX_bz_e</t>
+    <t xml:space="preserve">10.1128/AEM.01643-14</t>
   </si>
   <si>
     <t xml:space="preserve">BZ12DOX</t>
@@ -401,7 +401,7 @@
     <numFmt numFmtId="165" formatCode="0.000"/>
     <numFmt numFmtId="166" formatCode="General"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -451,6 +451,14 @@
       <color rgb="FF000000"/>
       <name val="JetBrains Mono"/>
       <family val="3"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -545,7 +553,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="25">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -586,11 +594,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -660,7 +672,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:M11"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
@@ -797,7 +809,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="2" t="s">
         <v>31</v>
       </c>
     </row>
@@ -817,8 +829,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AMJ36"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:N38"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="9" t="s">
@@ -851,7 +863,7 @@
       <c r="J1" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="K1" s="8" t="s">
+      <c r="K1" s="10" t="s">
         <v>33</v>
       </c>
       <c r="L1" s="8" t="s">
@@ -860,867 +872,932 @@
       <c r="M1" s="8" t="s">
         <v>35</v>
       </c>
-      <c r="AMJ1" s="0"/>
+      <c r="N1" s="8" t="s">
+        <v>36</v>
+      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="10" t="n">
+      <c r="A2" s="11" t="n">
         <v>0.73</v>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="11" t="n">
         <v>-7.3</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
-      <c r="I2" s="10"/>
-      <c r="J2" s="10"/>
-      <c r="K2" s="10" t="s">
-        <v>36</v>
-      </c>
+      <c r="C2" s="11"/>
+      <c r="D2" s="11"/>
+      <c r="E2" s="11"/>
+      <c r="F2" s="11"/>
+      <c r="G2" s="11"/>
+      <c r="H2" s="11"/>
+      <c r="I2" s="11"/>
+      <c r="J2" s="11"/>
+      <c r="K2" s="11"/>
       <c r="L2" s="11" t="s">
         <v>37</v>
       </c>
+      <c r="M2" s="12" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="10" t="n">
+      <c r="A3" s="11" t="n">
         <v>0.48</v>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="11" t="n">
         <v>-5.1</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
-      <c r="I3" s="10"/>
-      <c r="J3" s="10"/>
-      <c r="K3" s="10" t="s">
-        <v>36</v>
-      </c>
+      <c r="C3" s="11"/>
+      <c r="D3" s="11"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="11"/>
       <c r="L3" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="M3" s="2" t="s">
+      <c r="M3" s="12" t="s">
         <v>38</v>
       </c>
+      <c r="N3" s="2" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="n">
+      <c r="A4" s="11" t="n">
         <v>0.48</v>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="11" t="n">
         <v>-7</v>
       </c>
-      <c r="C4" s="10" t="n">
+      <c r="C4" s="11" t="n">
         <v>1.5</v>
       </c>
-      <c r="D4" s="10" t="n">
+      <c r="D4" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
-      <c r="I4" s="10"/>
-      <c r="J4" s="10"/>
-      <c r="K4" s="10" t="s">
-        <v>39</v>
-      </c>
-      <c r="L4" s="2" t="s">
+      <c r="E4" s="11"/>
+      <c r="F4" s="11"/>
+      <c r="G4" s="11"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+      <c r="J4" s="11"/>
+      <c r="K4" s="11"/>
+      <c r="L4" s="11" t="s">
         <v>40</v>
       </c>
+      <c r="M4" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="10" t="n">
+      <c r="A5" s="11" t="n">
         <v>0.57</v>
       </c>
-      <c r="B5" s="10" t="n">
+      <c r="B5" s="11" t="n">
         <v>-10.9</v>
       </c>
-      <c r="C5" s="10" t="n">
+      <c r="C5" s="11" t="n">
         <v>2.8</v>
       </c>
-      <c r="D5" s="10" t="n">
+      <c r="D5" s="11" t="n">
         <v>2.6</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
-      <c r="I5" s="10"/>
-      <c r="J5" s="10"/>
-      <c r="K5" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L5" s="2" t="s">
-        <v>40</v>
+      <c r="E5" s="11"/>
+      <c r="F5" s="11"/>
+      <c r="G5" s="11"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+      <c r="J5" s="11"/>
+      <c r="K5" s="11"/>
+      <c r="L5" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M5" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="10" t="n">
+      <c r="A6" s="11" t="n">
         <v>0.52</v>
       </c>
-      <c r="B6" s="10" t="n">
+      <c r="B6" s="11" t="n">
         <v>-19.1</v>
       </c>
-      <c r="C6" s="10" t="n">
+      <c r="C6" s="11" t="n">
         <v>5.1</v>
       </c>
-      <c r="D6" s="10" t="n">
+      <c r="D6" s="11" t="n">
         <v>7.2</v>
       </c>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
-      <c r="H6" s="10"/>
-      <c r="I6" s="10"/>
-      <c r="J6" s="10"/>
-      <c r="K6" s="10" t="s">
+      <c r="E6" s="11"/>
+      <c r="F6" s="11"/>
+      <c r="G6" s="11"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+      <c r="J6" s="11"/>
+      <c r="K6" s="11"/>
+      <c r="L6" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="M6" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="L6" s="2" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="10" t="n">
+      <c r="A7" s="11" t="n">
         <v>0.6</v>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="11" t="n">
         <v>-16.3</v>
       </c>
-      <c r="C7" s="10" t="n">
+      <c r="C7" s="11" t="n">
         <v>7.4</v>
       </c>
-      <c r="D7" s="10" t="n">
+      <c r="D7" s="11" t="n">
         <v>2.4</v>
       </c>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
-      <c r="H7" s="10"/>
-      <c r="I7" s="10"/>
-      <c r="J7" s="10"/>
-      <c r="K7" s="10" t="s">
-        <v>42</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>40</v>
+      <c r="E7" s="11"/>
+      <c r="F7" s="11"/>
+      <c r="G7" s="11"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+      <c r="J7" s="11"/>
+      <c r="K7" s="11"/>
+      <c r="L7" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="M7" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="10" t="n">
+      <c r="A8" s="11" t="n">
         <v>0.56</v>
       </c>
-      <c r="B8" s="10" t="n">
+      <c r="B8" s="11" t="n">
         <v>-6.31</v>
       </c>
-      <c r="C8" s="10" t="n">
+      <c r="C8" s="11" t="n">
         <v>1.75</v>
       </c>
-      <c r="D8" s="10" t="n">
+      <c r="D8" s="11" t="n">
         <v>0.53</v>
       </c>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
-      <c r="H8" s="10"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L8" s="2" t="s">
-        <v>43</v>
+      <c r="E8" s="11"/>
+      <c r="F8" s="11"/>
+      <c r="G8" s="11"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+      <c r="J8" s="11"/>
+      <c r="K8" s="11"/>
+      <c r="L8" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>44</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="10" t="n">
+      <c r="A9" s="11" t="n">
         <v>0.55</v>
       </c>
-      <c r="B9" s="10" t="n">
+      <c r="B9" s="11" t="n">
         <v>-6.14</v>
       </c>
-      <c r="C9" s="10" t="n">
+      <c r="C9" s="11" t="n">
         <v>2.13</v>
       </c>
-      <c r="D9" s="10" t="n">
+      <c r="D9" s="11" t="n">
         <v>0.44</v>
       </c>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
-      <c r="H9" s="10"/>
-      <c r="I9" s="10"/>
-      <c r="J9" s="10"/>
-      <c r="K9" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L9" s="2" t="s">
-        <v>44</v>
+      <c r="E9" s="11"/>
+      <c r="F9" s="11"/>
+      <c r="G9" s="11"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+      <c r="J9" s="11"/>
+      <c r="K9" s="11"/>
+      <c r="L9" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M9" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="10" t="n">
+      <c r="A10" s="11" t="n">
         <v>0.71</v>
       </c>
-      <c r="B10" s="12"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10" t="n">
+      <c r="B10" s="13"/>
+      <c r="C10" s="11"/>
+      <c r="D10" s="11"/>
+      <c r="E10" s="11" t="n">
         <v>-4.35</v>
       </c>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
-      <c r="H10" s="10"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L10" s="2" t="s">
-        <v>44</v>
+      <c r="F10" s="11"/>
+      <c r="G10" s="11"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+      <c r="J10" s="11"/>
+      <c r="K10" s="11"/>
+      <c r="L10" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M10" s="2" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="10" t="n">
+      <c r="A11" s="11" t="n">
         <v>0.72</v>
       </c>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
-      <c r="H11" s="10"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="10" t="n">
+      <c r="B11" s="11"/>
+      <c r="C11" s="11"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11"/>
+      <c r="F11" s="11"/>
+      <c r="G11" s="11"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+      <c r="J11" s="11" t="n">
         <v>-11.9</v>
       </c>
-      <c r="K11" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="L11" s="2" t="s">
+      <c r="K11" s="11"/>
+      <c r="L11" s="11" t="s">
         <v>46</v>
       </c>
       <c r="M11" s="2" t="s">
         <v>47</v>
       </c>
+      <c r="N11" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="10" t="n">
+      <c r="A12" s="11" t="n">
         <v>0.74</v>
       </c>
-      <c r="B12" s="10" t="n">
+      <c r="B12" s="11" t="n">
         <v>-5.7</v>
       </c>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
-      <c r="H12" s="10"/>
-      <c r="I12" s="10"/>
-      <c r="J12" s="10" t="n">
+      <c r="C12" s="11"/>
+      <c r="D12" s="11"/>
+      <c r="E12" s="11"/>
+      <c r="F12" s="11"/>
+      <c r="G12" s="11"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11" t="n">
         <v>-6.4</v>
       </c>
-      <c r="K12" s="10" t="s">
-        <v>45</v>
-      </c>
-      <c r="L12" s="2" t="s">
+      <c r="K12" s="11"/>
+      <c r="L12" s="11" t="s">
         <v>46</v>
       </c>
       <c r="M12" s="2" t="s">
         <v>47</v>
       </c>
+      <c r="N12" s="2" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="10" t="n">
+      <c r="A13" s="11" t="n">
         <v>0.48</v>
       </c>
-      <c r="B13" s="10" t="n">
+      <c r="B13" s="11" t="n">
         <v>-7</v>
       </c>
-      <c r="C13" s="10" t="n">
+      <c r="C13" s="11" t="n">
         <v>1.5</v>
       </c>
-      <c r="D13" s="10" t="n">
+      <c r="D13" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
-      <c r="H13" s="10"/>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10"/>
-      <c r="K13" s="12" t="s">
-        <v>39</v>
-      </c>
-      <c r="L13" s="2" t="s">
+      <c r="E13" s="11"/>
+      <c r="F13" s="11"/>
+      <c r="G13" s="11"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+      <c r="J13" s="11"/>
+      <c r="K13" s="11"/>
+      <c r="L13" s="13" t="s">
         <v>40</v>
       </c>
+      <c r="M13" s="2" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="10" t="n">
+      <c r="A14" s="11" t="n">
         <v>0.57</v>
       </c>
-      <c r="B14" s="10" t="n">
+      <c r="B14" s="11" t="n">
         <v>-10.9</v>
       </c>
-      <c r="C14" s="10" t="n">
+      <c r="C14" s="11" t="n">
         <v>2.8</v>
       </c>
-      <c r="D14" s="10" t="n">
+      <c r="D14" s="11" t="n">
         <v>2.6</v>
       </c>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
-      <c r="H14" s="10"/>
-      <c r="I14" s="10"/>
-      <c r="J14" s="10"/>
-      <c r="K14" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="L14" s="2" t="s">
-        <v>40</v>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+      <c r="L14" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="n">
+      <c r="A15" s="11" t="n">
         <v>0.52</v>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="11" t="n">
         <v>-19.1</v>
       </c>
-      <c r="C15" s="10" t="n">
+      <c r="C15" s="11" t="n">
         <v>5.1</v>
       </c>
-      <c r="D15" s="10" t="n">
+      <c r="D15" s="11" t="n">
         <v>7.2</v>
       </c>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
-      <c r="H15" s="10"/>
-      <c r="I15" s="10"/>
-      <c r="J15" s="10"/>
-      <c r="K15" s="12" t="s">
+      <c r="E15" s="11"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="11"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+      <c r="J15" s="11"/>
+      <c r="K15" s="11"/>
+      <c r="L15" s="13" t="s">
+        <v>42</v>
+      </c>
+      <c r="M15" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="L15" s="2" t="s">
-        <v>40</v>
-      </c>
     </row>
     <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+      <c r="A16" s="11" t="n">
         <v>0.61</v>
       </c>
-      <c r="B16" s="10" t="n">
+      <c r="B16" s="11" t="n">
         <v>-6</v>
       </c>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
-      <c r="H16" s="10"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="10"/>
-      <c r="K16" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L16" s="2" t="s">
-        <v>48</v>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+      <c r="L16" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="M16" s="2" t="s">
         <v>49</v>
       </c>
+      <c r="N16" s="2" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
+      <c r="A17" s="11" t="n">
         <v>0.2</v>
       </c>
-      <c r="B17" s="10" t="n">
+      <c r="B17" s="11" t="n">
         <v>-2</v>
       </c>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
-      <c r="H17" s="10"/>
-      <c r="I17" s="10"/>
-      <c r="J17" s="10"/>
-      <c r="K17" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L17" s="2" t="s">
-        <v>48</v>
+      <c r="C17" s="11"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+      <c r="J17" s="11"/>
+      <c r="K17" s="11"/>
+      <c r="L17" s="11" t="s">
+        <v>37</v>
       </c>
       <c r="M17" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
+      <c r="A18" s="11" t="n">
         <v>0.29</v>
       </c>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10" t="n">
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11" t="n">
         <v>-3.4</v>
       </c>
-      <c r="G18" s="10"/>
-      <c r="H18" s="10"/>
-      <c r="I18" s="10"/>
-      <c r="J18" s="10"/>
-      <c r="K18" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="L18" s="2" t="s">
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+      <c r="L18" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M18" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="n">
+      <c r="A19" s="11" t="n">
         <v>0.044</v>
       </c>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10" t="n">
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11" t="n">
         <f aca="false">-0.095/92.09382*1000</f>
         <v>-1.03155673203696</v>
       </c>
-      <c r="H19" s="10"/>
-      <c r="I19" s="10"/>
-      <c r="J19" s="10"/>
-      <c r="K19" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L19" s="2" t="s">
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+      <c r="J19" s="11"/>
+      <c r="K19" s="11"/>
+      <c r="L19" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M19" s="2" t="s">
+      <c r="N19" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="10" t="n">
+      <c r="A20" s="11" t="n">
         <v>0.066</v>
       </c>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10" t="n">
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11" t="n">
         <f aca="false">-0.137/92.09382*1000</f>
         <v>-1.48761339251646</v>
       </c>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L20" s="2" t="s">
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+      <c r="L20" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M20" s="2" t="s">
+      <c r="N20" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
+      <c r="A21" s="11" t="n">
         <v>0.088</v>
       </c>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10" t="n">
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11" t="n">
         <f aca="false">-0.168/92.09382*1000</f>
         <v>-1.82422664191799</v>
       </c>
-      <c r="H21" s="10"/>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10"/>
-      <c r="K21" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L21" s="2" t="s">
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+      <c r="J21" s="11"/>
+      <c r="K21" s="11"/>
+      <c r="L21" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M21" s="2" t="s">
+      <c r="N21" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="n">
+      <c r="A22" s="11" t="n">
         <v>0.109</v>
       </c>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10" t="n">
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11" t="n">
         <f aca="false">-0.215/92.09382*1000</f>
         <v>-2.33457576197838</v>
       </c>
-      <c r="H22" s="10"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="10"/>
-      <c r="K22" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L22" s="2" t="s">
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+      <c r="L22" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M22" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M22" s="2" t="s">
+      <c r="N22" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
+      <c r="A23" s="11" t="n">
         <v>0.12</v>
       </c>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10" t="n">
+      <c r="B23" s="11"/>
+      <c r="C23" s="11"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11"/>
+      <c r="F23" s="11"/>
+      <c r="G23" s="11" t="n">
         <f aca="false">-0.237/92.09382*1000</f>
         <v>-2.57346258413431</v>
       </c>
-      <c r="H23" s="10"/>
-      <c r="I23" s="10"/>
-      <c r="J23" s="10"/>
-      <c r="K23" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L23" s="2" t="s">
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+      <c r="J23" s="11"/>
+      <c r="K23" s="11"/>
+      <c r="L23" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M23" s="2" t="s">
+      <c r="N23" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10" t="n">
+      <c r="A24" s="11" t="n">
         <v>0.141</v>
       </c>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10" t="n">
+      <c r="B24" s="11"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11" t="n">
         <f aca="false">-0.288/92.09382*1000</f>
         <v>-3.12724567185941</v>
       </c>
-      <c r="H24" s="10"/>
-      <c r="I24" s="10"/>
-      <c r="J24" s="10"/>
-      <c r="K24" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L24" s="2" t="s">
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+      <c r="L24" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M24" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M24" s="2" t="s">
+      <c r="N24" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10" t="n">
+      <c r="A25" s="11" t="n">
         <v>0.19</v>
       </c>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10" t="n">
+      <c r="B25" s="11"/>
+      <c r="C25" s="11"/>
+      <c r="D25" s="11"/>
+      <c r="E25" s="11"/>
+      <c r="F25" s="11"/>
+      <c r="G25" s="11" t="n">
         <f aca="false">-0.39/92.09382*1000</f>
         <v>-4.23481184730962</v>
       </c>
-      <c r="H25" s="10"/>
-      <c r="I25" s="10"/>
-      <c r="J25" s="10"/>
-      <c r="K25" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L25" s="2" t="s">
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+      <c r="J25" s="11"/>
+      <c r="K25" s="11"/>
+      <c r="L25" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M25" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M25" s="2" t="s">
+      <c r="N25" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10" t="n">
+      <c r="A26" s="11" t="n">
         <v>0.21</v>
       </c>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10" t="n">
+      <c r="B26" s="11"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11" t="n">
         <f aca="false">-0.41/92.09382*1000</f>
         <v>-4.45198168563319</v>
       </c>
-      <c r="H26" s="10"/>
-      <c r="I26" s="10"/>
-      <c r="J26" s="10"/>
-      <c r="K26" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L26" s="2" t="s">
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+      <c r="L26" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="M26" s="2" t="s">
+      <c r="N26" s="2" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10" t="n">
+      <c r="A27" s="11" t="n">
         <v>0.05</v>
       </c>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
-      <c r="H27" s="10" t="n">
+      <c r="B27" s="11"/>
+      <c r="C27" s="11"/>
+      <c r="D27" s="11"/>
+      <c r="E27" s="11"/>
+      <c r="F27" s="11"/>
+      <c r="G27" s="11"/>
+      <c r="H27" s="11" t="n">
         <v>-1.3</v>
       </c>
-      <c r="I27" s="10"/>
-      <c r="J27" s="10"/>
-      <c r="K27" s="10" t="s">
-        <v>45</v>
-      </c>
+      <c r="I27" s="11"/>
+      <c r="J27" s="11"/>
+      <c r="K27" s="11"/>
       <c r="L27" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="M27" s="12" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10" t="n">
+      <c r="A28" s="11" t="n">
         <v>0.2</v>
       </c>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
-      <c r="H28" s="10" t="n">
+      <c r="B28" s="11"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11" t="n">
         <v>-4.6</v>
       </c>
-      <c r="I28" s="10"/>
-      <c r="J28" s="10"/>
-      <c r="K28" s="10" t="s">
-        <v>45</v>
-      </c>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
       <c r="L28" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="M28" s="12" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10" t="n">
+      <c r="A29" s="11" t="n">
         <v>0.3</v>
       </c>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
-      <c r="H29" s="10" t="n">
+      <c r="B29" s="11"/>
+      <c r="C29" s="11"/>
+      <c r="D29" s="11"/>
+      <c r="E29" s="11"/>
+      <c r="F29" s="11"/>
+      <c r="G29" s="11"/>
+      <c r="H29" s="11" t="n">
         <v>-5.8</v>
       </c>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10"/>
-      <c r="K29" s="10" t="s">
-        <v>45</v>
-      </c>
+      <c r="I29" s="11"/>
+      <c r="J29" s="11"/>
+      <c r="K29" s="11"/>
       <c r="L29" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="M29" s="12" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10" t="n">
+      <c r="A30" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
-      <c r="H30" s="10" t="n">
+      <c r="B30" s="11"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11" t="n">
         <v>-7.3</v>
       </c>
-      <c r="I30" s="10"/>
-      <c r="J30" s="10"/>
-      <c r="K30" s="10" t="s">
-        <v>45</v>
-      </c>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
       <c r="L30" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="M30" s="12" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10" t="n">
+      <c r="A31" s="11" t="n">
         <v>0.58</v>
       </c>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
-      <c r="H31" s="10" t="n">
+      <c r="B31" s="11"/>
+      <c r="C31" s="11"/>
+      <c r="D31" s="11"/>
+      <c r="E31" s="11"/>
+      <c r="F31" s="11"/>
+      <c r="G31" s="11"/>
+      <c r="H31" s="11" t="n">
         <v>-10.2</v>
       </c>
-      <c r="I31" s="10"/>
-      <c r="J31" s="10"/>
-      <c r="K31" s="10" t="s">
-        <v>45</v>
-      </c>
+      <c r="I31" s="11"/>
+      <c r="J31" s="11"/>
+      <c r="K31" s="11"/>
       <c r="L31" s="11" t="s">
+        <v>46</v>
+      </c>
+      <c r="M31" s="12" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10" t="n">
+      <c r="A32" s="11" t="n">
         <v>0.25</v>
       </c>
-      <c r="B32" s="10" t="n">
+      <c r="B32" s="11" t="n">
         <v>-4.79</v>
       </c>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
-      <c r="H32" s="10"/>
-      <c r="I32" s="10"/>
-      <c r="J32" s="10"/>
-      <c r="K32" s="10" t="s">
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+      <c r="J32" s="11"/>
+      <c r="K32" s="11"/>
+      <c r="L32" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="L32" s="2" t="s">
+      <c r="M32" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M32" s="2" t="s">
+      <c r="N32" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10" t="n">
+      <c r="A33" s="11" t="n">
         <v>0.15</v>
       </c>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
-      <c r="H33" s="10"/>
-      <c r="I33" s="10" t="n">
+      <c r="B33" s="11"/>
+      <c r="C33" s="11"/>
+      <c r="D33" s="11"/>
+      <c r="E33" s="11"/>
+      <c r="F33" s="11"/>
+      <c r="G33" s="11"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11" t="n">
         <v>-0.85</v>
       </c>
-      <c r="J33" s="10"/>
-      <c r="K33" s="10" t="s">
+      <c r="J33" s="11"/>
+      <c r="K33" s="11"/>
+      <c r="L33" s="11" t="s">
         <v>56</v>
       </c>
-      <c r="L33" s="2" t="s">
+      <c r="M33" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="M33" s="2" t="s">
+      <c r="N33" s="2" t="s">
         <v>58</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="10" t="n">
+      <c r="A34" s="11" t="n">
         <v>0.68</v>
       </c>
-      <c r="B34" s="10" t="n">
+      <c r="B34" s="11" t="n">
         <v>-6.49</v>
       </c>
-      <c r="C34" s="10"/>
-      <c r="D34" s="10"/>
-      <c r="E34" s="10"/>
-      <c r="F34" s="10"/>
-      <c r="G34" s="10"/>
-      <c r="H34" s="10"/>
-      <c r="I34" s="10"/>
-      <c r="J34" s="10"/>
-      <c r="K34" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L34" s="2" t="s">
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="11"/>
+      <c r="K34" s="11"/>
+      <c r="L34" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M34" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="10" t="n">
+      <c r="A35" s="11" t="n">
         <v>0.72</v>
       </c>
-      <c r="B35" s="10"/>
-      <c r="C35" s="10"/>
-      <c r="D35" s="10"/>
-      <c r="E35" s="10" t="n">
+      <c r="B35" s="11"/>
+      <c r="C35" s="11"/>
+      <c r="D35" s="11"/>
+      <c r="E35" s="11" t="n">
         <v>-4.81</v>
       </c>
-      <c r="F35" s="10"/>
-      <c r="G35" s="10"/>
-      <c r="H35" s="10"/>
-      <c r="I35" s="10"/>
-      <c r="J35" s="10"/>
-      <c r="K35" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L35" s="2" t="s">
+      <c r="F35" s="11"/>
+      <c r="G35" s="11"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+      <c r="J35" s="11"/>
+      <c r="K35" s="11"/>
+      <c r="L35" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M35" s="2" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="10" t="n">
+      <c r="A36" s="11" t="n">
         <v>0.46</v>
       </c>
-      <c r="B36" s="10"/>
-      <c r="C36" s="10"/>
-      <c r="D36" s="10"/>
-      <c r="E36" s="10"/>
-      <c r="F36" s="10"/>
-      <c r="G36" s="10" t="n">
+      <c r="B36" s="11"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11" t="n">
         <v>-3.95</v>
       </c>
-      <c r="H36" s="10"/>
-      <c r="I36" s="10"/>
-      <c r="J36" s="10"/>
-      <c r="K36" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="L36" s="2" t="s">
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+      <c r="J36" s="11"/>
+      <c r="K36" s="11"/>
+      <c r="L36" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="M36" s="2" t="s">
         <v>59</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="I37" s="0" t="n">
+        <v>-1.62</v>
+      </c>
+      <c r="L37" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="M37" s="2" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="0" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="K38" s="0" t="n">
+        <v>-1.96</v>
+      </c>
+      <c r="L38" s="0" t="s">
+        <v>37</v>
+      </c>
+      <c r="M38" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -1740,11 +1817,11 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AK3"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
-        <v>60</v>
+        <v>33</v>
       </c>
       <c r="B1" s="8" t="s">
         <v>61</v>
@@ -1849,10 +1926,10 @@
         <v>4</v>
       </c>
       <c r="AJ1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="8" t="s">
         <v>34</v>
-      </c>
-      <c r="AK1" s="8" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1868,13 +1945,13 @@
       <c r="D2" s="2" t="n">
         <v>3.41</v>
       </c>
-      <c r="E2" s="13" t="n">
+      <c r="E2" s="14" t="n">
         <v>3.41</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>3.41</v>
       </c>
-      <c r="G2" s="13" t="n">
+      <c r="G2" s="14" t="n">
         <v>3.41</v>
       </c>
       <c r="H2" s="2" t="n">
@@ -1883,22 +1960,22 @@
       <c r="I2" s="2" t="n">
         <v>3.41</v>
       </c>
-      <c r="J2" s="13" t="n">
+      <c r="J2" s="14" t="n">
         <v>4.07</v>
       </c>
-      <c r="K2" s="13" t="n">
+      <c r="K2" s="14" t="n">
         <v>4.07</v>
       </c>
-      <c r="L2" s="13" t="n">
+      <c r="L2" s="14" t="n">
         <v>4.07</v>
       </c>
       <c r="M2" s="2" t="n">
         <v>3.41</v>
       </c>
-      <c r="N2" s="13" t="n">
+      <c r="N2" s="14" t="n">
         <v>7.15</v>
       </c>
-      <c r="O2" s="13" t="n">
+      <c r="O2" s="14" t="n">
         <v>7.15</v>
       </c>
       <c r="P2" s="2" t="n">
@@ -1913,10 +1990,10 @@
       <c r="S2" s="2" t="n">
         <v>0.66</v>
       </c>
-      <c r="T2" s="14" t="n">
+      <c r="T2" s="15" t="n">
         <v>0.33</v>
       </c>
-      <c r="U2" s="14" t="n">
+      <c r="U2" s="15" t="n">
         <v>0.33</v>
       </c>
       <c r="V2" s="2" t="n">
@@ -1928,13 +2005,13 @@
       <c r="X2" s="2" t="n">
         <v>0.67</v>
       </c>
-      <c r="Y2" s="15" t="n">
+      <c r="Y2" s="16" t="n">
         <v>0.35</v>
       </c>
-      <c r="Z2" s="15" t="n">
+      <c r="Z2" s="16" t="n">
         <v>0.35</v>
       </c>
-      <c r="AA2" s="15" t="n">
+      <c r="AA2" s="16" t="n">
         <v>0.35</v>
       </c>
       <c r="AB2" s="2" t="n">
@@ -1961,11 +2038,11 @@
       <c r="AI2" s="2" t="n">
         <v>0.2</v>
       </c>
-      <c r="AJ2" s="11" t="s">
+      <c r="AJ2" s="12" t="s">
         <v>94</v>
       </c>
-      <c r="AK2" s="0" t="s">
-        <v>36</v>
+      <c r="AK2" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2062,14 +2139,14 @@
       <c r="AG3" s="2" t="n">
         <v>0.05</v>
       </c>
-      <c r="AI3" s="0" t="n">
+      <c r="AI3" s="2" t="n">
         <v>0.1</v>
       </c>
       <c r="AJ3" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="AK3" s="0" t="s">
-        <v>36</v>
+      <c r="AK3" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2089,7 +2166,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AQ7"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -2101,106 +2178,106 @@
       <c r="C1" s="8" t="s">
         <v>97</v>
       </c>
-      <c r="D1" s="16" t="s">
+      <c r="D1" s="17" t="s">
         <v>98</v>
       </c>
-      <c r="E1" s="17" t="s">
+      <c r="E1" s="18" t="s">
         <v>99</v>
       </c>
-      <c r="F1" s="17" t="s">
+      <c r="F1" s="18" t="s">
         <v>100</v>
       </c>
-      <c r="G1" s="17" t="s">
+      <c r="G1" s="18" t="s">
         <v>101</v>
       </c>
-      <c r="H1" s="17" t="s">
+      <c r="H1" s="18" t="s">
         <v>102</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="17" t="s">
         <v>88</v>
       </c>
-      <c r="J1" s="17" t="s">
+      <c r="J1" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="K1" s="18" t="s">
+      <c r="K1" s="19" t="s">
         <v>90</v>
       </c>
-      <c r="L1" s="16" t="s">
+      <c r="L1" s="17" t="s">
         <v>103</v>
       </c>
-      <c r="M1" s="17" t="s">
+      <c r="M1" s="18" t="s">
         <v>104</v>
       </c>
-      <c r="N1" s="17" t="s">
+      <c r="N1" s="18" t="s">
         <v>105</v>
       </c>
-      <c r="O1" s="17" t="s">
+      <c r="O1" s="18" t="s">
         <v>106</v>
       </c>
-      <c r="P1" s="17" t="s">
+      <c r="P1" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="Q1" s="17" t="s">
+      <c r="Q1" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="R1" s="17" t="s">
+      <c r="R1" s="18" t="s">
         <v>93</v>
       </c>
-      <c r="S1" s="18" t="s">
+      <c r="S1" s="19" t="s">
         <v>91</v>
       </c>
-      <c r="T1" s="18" t="s">
+      <c r="T1" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="U1" s="16" t="s">
+      <c r="U1" s="17" t="s">
         <v>86</v>
       </c>
-      <c r="V1" s="17" t="s">
+      <c r="V1" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="W1" s="17" t="s">
+      <c r="W1" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="X1" s="17" t="s">
+      <c r="X1" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="Y1" s="18" t="s">
+      <c r="Y1" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="Z1" s="16" t="s">
+      <c r="Z1" s="17" t="s">
         <v>77</v>
       </c>
-      <c r="AA1" s="17" t="s">
+      <c r="AA1" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="AB1" s="17" t="s">
+      <c r="AB1" s="18" t="s">
         <v>110</v>
       </c>
-      <c r="AC1" s="17" t="s">
+      <c r="AC1" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="AD1" s="17" t="s">
+      <c r="AD1" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="AE1" s="17" t="s">
+      <c r="AE1" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="AF1" s="17" t="s">
+      <c r="AF1" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="AG1" s="17" t="s">
+      <c r="AG1" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="AH1" s="17" t="s">
+      <c r="AH1" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="AI1" s="17" t="s">
+      <c r="AI1" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="AJ1" s="17" t="s">
+      <c r="AJ1" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="AK1" s="18" t="s">
+      <c r="AK1" s="19" t="s">
         <v>75</v>
       </c>
       <c r="AL1" s="8" t="s">
@@ -2216,170 +2293,170 @@
         <v>4</v>
       </c>
       <c r="AP1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AQ1" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="AQ1" s="8" t="s">
-        <v>33</v>
-      </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="n">
+      <c r="A2" s="20" t="n">
         <f aca="false">-100/100*6.14</f>
         <v>-6.14</v>
       </c>
-      <c r="B2" s="19" t="n">
+      <c r="B2" s="20" t="n">
         <f aca="false">90/100*6.14</f>
         <v>5.526</v>
       </c>
-      <c r="C2" s="19" t="n">
+      <c r="C2" s="20" t="n">
         <f aca="false">12/100*6.14</f>
         <v>0.7368</v>
       </c>
-      <c r="D2" s="20" t="n">
+      <c r="D2" s="21" t="n">
         <f aca="false">10/100*6.14</f>
         <v>0.614</v>
       </c>
-      <c r="E2" s="21" t="n">
+      <c r="E2" s="22" t="n">
         <f aca="false">19/100*6.14</f>
         <v>1.1666</v>
       </c>
-      <c r="F2" s="21" t="n">
+      <c r="F2" s="22" t="n">
         <f aca="false">19/100*6.14</f>
         <v>1.1666</v>
       </c>
-      <c r="G2" s="19" t="n">
+      <c r="G2" s="20" t="n">
         <f aca="false">99/100*6.14</f>
         <v>6.0786</v>
       </c>
-      <c r="H2" s="19" t="n">
+      <c r="H2" s="20" t="n">
         <f aca="false">99/100*6.14</f>
         <v>6.0786</v>
       </c>
-      <c r="I2" s="22" t="n">
+      <c r="I2" s="23" t="n">
         <f aca="false">8/100*6.14</f>
         <v>0.4912</v>
       </c>
-      <c r="J2" s="19" t="n">
+      <c r="J2" s="20" t="n">
         <f aca="false">8/100*6.14</f>
         <v>0.4912</v>
       </c>
-      <c r="K2" s="23" t="n">
+      <c r="K2" s="24" t="n">
         <f aca="false">9/100*6.14</f>
         <v>0.5526</v>
       </c>
-      <c r="L2" s="22" t="n">
+      <c r="L2" s="23" t="n">
         <f aca="false">78/100*6.14</f>
         <v>4.7892</v>
       </c>
-      <c r="M2" s="19" t="n">
+      <c r="M2" s="20" t="n">
         <f aca="false">12/100*6.14</f>
         <v>0.7368</v>
       </c>
-      <c r="N2" s="19" t="n">
+      <c r="N2" s="20" t="n">
         <f aca="false">12/100*6.14</f>
         <v>0.7368</v>
       </c>
-      <c r="O2" s="21" t="n">
+      <c r="O2" s="22" t="n">
         <f aca="false">10/100*6.14</f>
         <v>0.614</v>
       </c>
-      <c r="P2" s="19" t="n">
+      <c r="P2" s="20" t="n">
         <f aca="false">7/100*6.14</f>
         <v>0.4298</v>
       </c>
-      <c r="Q2" s="19" t="n">
+      <c r="Q2" s="20" t="n">
         <f aca="false">2/100*6.14</f>
         <v>0.1228</v>
       </c>
-      <c r="R2" s="19" t="n">
+      <c r="R2" s="20" t="n">
         <f aca="false">2/100*6.14</f>
         <v>0.1228</v>
       </c>
-      <c r="S2" s="23" t="n">
+      <c r="S2" s="24" t="n">
         <f aca="false">2/100*6.14</f>
         <v>0.1228</v>
       </c>
-      <c r="T2" s="23"/>
-      <c r="U2" s="22" t="n">
+      <c r="T2" s="24"/>
+      <c r="U2" s="23" t="n">
         <f aca="false">83/100*6.14</f>
         <v>5.0962</v>
       </c>
-      <c r="V2" s="19" t="n">
+      <c r="V2" s="20" t="n">
         <f aca="false">83/100*6.14</f>
         <v>5.0962</v>
       </c>
-      <c r="W2" s="19" t="n">
+      <c r="W2" s="20" t="n">
         <f aca="false">71/100*6.14</f>
         <v>4.3594</v>
       </c>
-      <c r="X2" s="19" t="n">
+      <c r="X2" s="20" t="n">
         <f aca="false">71/100*6.14</f>
         <v>4.3594</v>
       </c>
-      <c r="Y2" s="23" t="n">
+      <c r="Y2" s="24" t="n">
         <f aca="false">63/100*6.14</f>
         <v>3.8682</v>
       </c>
-      <c r="Z2" s="22" t="n">
+      <c r="Z2" s="23" t="n">
         <f aca="false">109/100*6.14</f>
         <v>6.6926</v>
       </c>
-      <c r="AA2" s="19" t="n">
+      <c r="AA2" s="20" t="n">
         <f aca="false">89/100*6.14</f>
         <v>5.4646</v>
       </c>
-      <c r="AB2" s="19" t="n">
+      <c r="AB2" s="20" t="n">
         <f aca="false">72/100*6.14</f>
         <v>4.4208</v>
       </c>
-      <c r="AC2" s="19" t="n">
+      <c r="AC2" s="20" t="n">
         <f aca="false">2/100*6.14</f>
         <v>0.1228</v>
       </c>
-      <c r="AD2" s="19" t="n">
+      <c r="AD2" s="20" t="n">
         <f aca="false">89/100*6.14</f>
         <v>5.4646</v>
       </c>
-      <c r="AE2" s="19" t="n">
+      <c r="AE2" s="20" t="n">
         <f aca="false">89/100*6.14</f>
         <v>5.4646</v>
       </c>
-      <c r="AF2" s="19" t="n">
+      <c r="AF2" s="20" t="n">
         <f aca="false">89/100*6.14</f>
         <v>5.4646</v>
       </c>
-      <c r="AG2" s="19" t="n">
+      <c r="AG2" s="20" t="n">
         <f aca="false">76/100*6.14</f>
         <v>4.6664</v>
       </c>
-      <c r="AH2" s="19" t="n">
+      <c r="AH2" s="20" t="n">
         <f aca="false">76/100*6.14</f>
         <v>4.6664</v>
       </c>
-      <c r="AI2" s="19" t="n">
+      <c r="AI2" s="20" t="n">
         <f aca="false">76/100*6.14</f>
         <v>4.6664</v>
       </c>
-      <c r="AJ2" s="19" t="n">
+      <c r="AJ2" s="20" t="n">
         <f aca="false">76/100*6.14</f>
         <v>4.6664</v>
       </c>
-      <c r="AK2" s="23" t="n">
+      <c r="AK2" s="24" t="n">
         <f aca="false">33/100*6.14</f>
         <v>2.0262</v>
       </c>
-      <c r="AL2" s="19" t="n">
+      <c r="AL2" s="20" t="n">
         <f aca="false">44/100*6.14</f>
         <v>2.7016</v>
       </c>
-      <c r="AO2" s="0" t="n">
+      <c r="AO2" s="2" t="n">
         <v>0.55</v>
       </c>
-      <c r="AP2" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="AQ2" s="0" t="s">
-        <v>36</v>
+      <c r="AP2" s="12" t="s">
+        <v>45</v>
+      </c>
+      <c r="AQ2" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2475,14 +2552,14 @@
         <f aca="false">10/100*5.7</f>
         <v>0.57</v>
       </c>
-      <c r="AO3" s="0" t="n">
+      <c r="AO3" s="2" t="n">
         <v>0.57</v>
       </c>
-      <c r="AP3" s="11" t="s">
+      <c r="AP3" s="12" t="s">
         <v>113</v>
       </c>
-      <c r="AQ3" s="0" t="s">
-        <v>36</v>
+      <c r="AQ3" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2579,14 +2656,14 @@
         <f aca="false">18/100*5.2</f>
         <v>0.936</v>
       </c>
-      <c r="AO4" s="0" t="n">
+      <c r="AO4" s="2" t="n">
         <v>0.48</v>
       </c>
-      <c r="AP4" s="11" t="s">
+      <c r="AP4" s="12" t="s">
         <v>114</v>
       </c>
-      <c r="AQ4" s="0" t="s">
-        <v>39</v>
+      <c r="AQ4" s="2" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2683,14 +2760,14 @@
         <f aca="false">16/100*6.5</f>
         <v>1.04</v>
       </c>
-      <c r="AO5" s="0" t="n">
+      <c r="AO5" s="2" t="n">
         <v>0.52</v>
       </c>
-      <c r="AP5" s="11" t="s">
+      <c r="AP5" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="AQ5" s="0" t="s">
-        <v>41</v>
+      <c r="AQ5" s="2" t="s">
+        <v>42</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2803,14 +2880,14 @@
         <f aca="false">50/100*6.01</f>
         <v>3.005</v>
       </c>
-      <c r="AO6" s="0" t="n">
+      <c r="AO6" s="2" t="n">
         <v>0.61</v>
       </c>
-      <c r="AP6" s="11" t="s">
+      <c r="AP6" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="AQ6" s="0" t="s">
-        <v>36</v>
+      <c r="AQ6" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2924,14 +3001,14 @@
         <f aca="false">54/100*2.01</f>
         <v>1.0854</v>
       </c>
-      <c r="AO7" s="0" t="n">
+      <c r="AO7" s="2" t="n">
         <v>0.2</v>
       </c>
-      <c r="AP7" s="11" t="s">
+      <c r="AP7" s="12" t="s">
         <v>117</v>
       </c>
-      <c r="AQ7" s="0" t="s">
-        <v>36</v>
+      <c r="AQ7" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -2951,7 +3028,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AG2"/>
-  <sheetFormatPr defaultColWidth="11.58984375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" s="8" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="8" t="s">
@@ -3048,10 +3125,10 @@
         <v>81</v>
       </c>
       <c r="AF1" s="8" t="s">
+        <v>35</v>
+      </c>
+      <c r="AG1" s="8" t="s">
         <v>34</v>
-      </c>
-      <c r="AG1" s="8" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3151,8 +3228,8 @@
       <c r="AF2" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="AG2" s="0" t="s">
-        <v>36</v>
+      <c r="AG2" s="2" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>